<commit_message>
QD-13: chuẩn hoá 3 dạng nghe theo record mẫu JFT (q07–q09) – không người dẫn, độ dài lượt, tranh người nói; viết lại 12 câu nghe DF-01; kiểm tra tự động; mô phỏng 14/14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011epdNWjc77FA9dxPqBsa8Z
</commit_message>
<xml_diff>
--- a/exports/DF-01_LMS_import.xlsx
+++ b/exports/DF-01_LMS_import.xlsx
@@ -1567,7 +1567,7 @@
       <c r="B26" t="inlineStr">
         <is>
           <t>Nghe hội thoại và chọn tranh đúng.
-Ở căng tin, một người phụ nữ và một người đàn ông đang nói chuyện.
+Bạn sẽ nghe hai đồng nghiệp nói chuyện về bữa sáng ở công ty.
 Người đàn ông thường ăn gì vào bữa sáng?</t>
         </is>
       </c>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>"いつも パンと たまごです" → bánh mì và trứng. Hôm nay không ăn gì là chi tiết nhiễu.</t>
+          <t>"パンと たまごです。コーヒーも 飲みます" → bánh mì, trứng, cà phê. Cơm thì あまり食べません; chuối là đồng nghiệp mời hôm nay.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1618,8 +1618,8 @@
       <c r="B27" t="inlineStr">
         <is>
           <t>Nghe hội thoại và chọn tranh đúng.
-Hai đồng nghiệp nói chuyện về ngày nghỉ.
-Bây giờ người phụ nữ thích làm gì vào ngày nghỉ?</t>
+Bạn sẽ nghe hai đồng nghiệp nói chuyện về ngày nghỉ.
+Bây giờ vào ngày nghỉ, người phụ nữ thường làm gì?</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>"今は りょうりを するのが すきです" → nấu ăn. Tennis là trước đây.</t>
+          <t>"最近は 家で 料理を するのが 好きです。週末は いつも ケーキを 作って います" → làm bánh ở nhà. Tennis là trước đây.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1669,16 +1669,16 @@
       <c r="B28" t="inlineStr">
         <is>
           <t>Nghe hội thoại và chọn tranh đúng.
-Hai người bạn hẹn nhau đi mua sắm.
+Bạn sẽ nghe hai người bạn hẹn nhau đi mua sắm.
 Hai người sẽ gặp nhau lúc mấy giờ?</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10 giờ không được (ちょっと…), chốt 11 giờ.</t>
+          <t>10 giờ thì ちょっと… vì có lớp đến 12 giờ; chốt "1時に 駅の 前で".</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1720,7 +1720,7 @@
       <c r="B29" t="inlineStr">
         <is>
           <t>Nghe hội thoại và chọn tranh đúng.
-Ở văn phòng, đồng nghiệp hỏi thăm một người đàn ông.
+Bạn sẽ nghe một người phụ nữ hỏi thăm đồng nghiệp ở công ty.
 Người đàn ông bị làm sao?</t>
         </is>
       </c>
@@ -1729,7 +1729,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>"のどが いたくて… ねつは ありません" → đau họng.</t>
+          <t>"きのうの よるから のどが いたいんです"; không sốt, không đau đầu.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1771,8 +1771,8 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>Nghe hội thoại và chọn tranh đúng.
-Ở cửa hàng đồ ăn nhanh, khách đang gọi món.
-Cuối cùng khách gọi gì?</t>
+Bạn sẽ nghe một người đàn ông gọi món ở cửa hàng hamburger.
+Cuối cùng người đàn ông gọi gì?</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Khách gọi hamburger + nước ép cỡ M, rồi đổi nước ép sang cà phê (ジュースじゃなくて、コーヒーに) → hamburger + cà phê.</t>
+          <t>Khách gọi nước cam cỡ M rồi đổi: "ジュースじゃなくて、コーヒーに して ください" → hamburger + cà phê cỡ M.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1822,7 +1822,7 @@
       <c r="B31" t="inlineStr">
         <is>
           <t>Nghe hội thoại và chọn tranh đúng.
-Một người hỏi đường trên phố.
+Bạn sẽ nghe một người đàn ông hỏi đường đến bưu điện.
 Bưu điện ở đâu?</t>
         </is>
       </c>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Đi thẳng, rẽ trái ở góc ngân hàng, bưu điện cạnh siêu thị.</t>
+          <t>"まっすぐ 行って… 銀行の かどを 左に まがって… スーパーの となり".</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1873,8 +1873,8 @@
       <c r="B32" t="inlineStr">
         <is>
           <t>Nghe hội thoại và chọn tranh đúng.
-Ở hiệu thuốc, dược sĩ giải thích cách uống thuốc.
-Uống thuốc khi nào?</t>
+Bạn sẽ nghe dược sĩ giải thích cách uống thuốc cho một người đàn ông ở hiệu thuốc.
+Người đàn ông uống thuốc khi nào?</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>"ごはんを 食べた あとで" và không uống trước khi ngủ.</t>
+          <t>"ごはんを 食べた あとで 飲んで ください"; không uống trước khi ngủ.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1924,8 +1924,8 @@
       <c r="B33" t="inlineStr">
         <is>
           <t>Nghe hội thoại và chọn tranh đúng.
-Ở tiệm cắt tóc, khách nói kiểu tóc mong muốn.
-Khách muốn cắt tóc thế nào?</t>
+Bạn sẽ nghe một người phụ nữ nói kiểu tóc mong muốn ở tiệm cắt tóc.
+Người phụ nữ muốn cắt tóc thế nào?</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Tóc mái cắt ngắn, phía sau không cắt nhiều.</t>
+          <t>"前髪を 短く… 目の 上ぐらいまで"; "うしろは 長いままが いいです".</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1975,8 +1975,10 @@
       <c r="B34" t="inlineStr">
         <is>
           <t>Nghe và trả lời câu hỏi (1) và (2).
-Ở nhà ga có thông báo.
-(1) Tàu bị chậm bao lâu?</t>
+Bạn sẽ nghe thông báo của nhân viên nhà ga.
+(1) Tàu bị chậm khoảng bao lâu?
+(2) Tàu đi Tokyo xuất phát từ sân ga số mấy?
+(1) Tàu bị chậm khoảng bao lâu?</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1984,7 +1986,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>"電車が 20分 おくれて います" → 20 phút.</t>
+          <t>"電車が 20分ぐらい おくれて います" → 20 phút.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2026,8 +2028,10 @@
       <c r="B35" t="inlineStr">
         <is>
           <t>Nghe và trả lời câu hỏi (1) và (2).
-Ở nhà ga có thông báo.
-(2) Tàu xuất phát từ sân ga số mấy?</t>
+Bạn sẽ nghe thông báo của nhân viên nhà ga.
+(1) Tàu bị chậm khoảng bao lâu?
+(2) Tàu đi Tokyo xuất phát từ sân ga số mấy?
+(2) Tàu đi Tokyo xuất phát từ sân ga số mấy?</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2035,7 +2039,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>"3番線ではなく、5番線から" → sân ga số 5.</t>
+          <t>"いつもの 3番線ではなく、5番線から 出発します" → sân ga 5.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2077,16 +2081,18 @@
       <c r="B36" t="inlineStr">
         <is>
           <t>Nghe và trả lời câu hỏi (1) và (2).
-Ở công ty, người phụ trách giải thích buổi diễn tập phòng chống động đất.
+Bạn sẽ nghe người phụ trách ở công ty giải thích việc cần làm khi có động đất trong buổi diễn tập.
+(1) Khi có động đất, đầu tiên phải làm gì?
+(2) Sau đó tập trung ở đâu?
 (1) Khi có động đất, đầu tiên phải làm gì?</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>"まず 机の 下に 入って ください" → chui xuống gầm bàn.</t>
+          <t>"まず 机の 下に 入って、頭を 守って ください".</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2128,16 +2134,18 @@
       <c r="B37" t="inlineStr">
         <is>
           <t>Nghe và trả lời câu hỏi (1) và (2).
-Ở công ty, người phụ trách giải thích buổi diễn tập phòng chống động đất.
-(2) Khi hết rung, xuống tầng 1 bằng gì?</t>
+Bạn sẽ nghe người phụ trách ở công ty giải thích việc cần làm khi có động đất trong buổi diễn tập.
+(1) Khi có động đất, đầu tiên phải làm gì?
+(2) Sau đó tập trung ở đâu?
+(2) Sau đó tập trung ở đâu?</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>"エレベーターは 使わないで、かいだんで" → cầu thang bộ.</t>
+          <t>"会社の 前の 公園に 集まって ください"; không đến bãi đỗ xe.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">

</xml_diff>

<commit_message>
DF-01: đóng khung BÀI ĐỌC cho câu 4-1/4-2 trong file LMS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011epdNWjc77FA9dxPqBsa8Z
</commit_message>
<xml_diff>
--- a/exports/DF-01_LMS_import.xlsx
+++ b/exports/DF-01_LMS_import.xlsx
@@ -2183,10 +2183,12 @@
       <c r="B38" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 たなかさん、おはようございます。グエンです。
 きのうの よるから ねつが あって、きょうは 会社を 休みたいです。
 あしたは 来られると 思います。
 よろしく おねがいします。
+━━━━━━━━━━━━━━━━━━
 (1) グエンさんは どうして 会社を 休みますか。</t>
         </is>
       </c>
@@ -2229,10 +2231,12 @@
       <c r="B39" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 たなかさん、おはようございます。グエンです。
 きのうの よるから ねつが あって、きょうは 会社を 休みたいです。
 あしたは 来られると 思います。
 よろしく おねがいします。
+━━━━━━━━━━━━━━━━━━
 (2) グエンさんは いつ 会社に 来られると 思って いますか。</t>
         </is>
       </c>
@@ -2275,10 +2279,12 @@
       <c r="B40" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 日曜日、家族と すいぞくかんに 行きました。
 イルカの ショーが とても おもしろかったです。
 むすこは ペンギンが いちばん 好きだと 言って いました。
 また 行きたいです。
+━━━━━━━━━━━━━━━━━━
 (1) この 人は 日曜日に だれと 出かけましたか。</t>
         </is>
       </c>
@@ -2321,10 +2327,12 @@
       <c r="B41" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 日曜日、家族と すいぞくかんに 行きました。
 イルカの ショーが とても おもしろかったです。
 むすこは ペンギンが いちばん 好きだと 言って いました。
 また 行きたいです。
+━━━━━━━━━━━━━━━━━━
 (2) むすこは 何が いちばん 好きですか。</t>
         </is>
       </c>
@@ -2367,11 +2375,13 @@
       <c r="B42" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 リンさんへ
 10時までに この はこを 2階の そうこに 運んで ください。
 そのあと、会議室の いすを ならべて ください。
 11時から 会議が あります。
 山本
+━━━━━━━━━━━━━━━━━━
 (1) リンさんは 最初に 何を しますか。</t>
         </is>
       </c>
@@ -2414,11 +2424,13 @@
       <c r="B43" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 リンさんへ
 10時までに この はこを 2階の そうこに 運んで ください。
 そのあと、会議室の いすを ならべて ください。
 11時から 会議が あります。
 山本
+━━━━━━━━━━━━━━━━━━
 (2) 会議は 何時から ですか。</t>
         </is>
       </c>
@@ -2461,6 +2473,7 @@
       <c r="B44" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 ランチメニュー
 カレー　650円
 ラーメン　700円
@@ -2468,6 +2481,7 @@
 サラダ　200円
 ドリンク（コーヒー・こうちゃ）　150円
 ※ランチは 11:00～14:00
+━━━━━━━━━━━━━━━━━━
 (1) 600円で 食べられる ものは どれですか。</t>
         </is>
       </c>
@@ -2510,6 +2524,7 @@
       <c r="B45" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 ランチメニュー
 カレー　650円
 ラーメン　700円
@@ -2517,6 +2532,7 @@
 サラダ　200円
 ドリンク（コーヒー・こうちゃ）　150円
 ※ランチは 11:00～14:00
+━━━━━━━━━━━━━━━━━━
 (2) ランチは 何時まで ですか。</t>
         </is>
       </c>
@@ -2559,12 +2575,14 @@
       <c r="B46" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 ゴミの 出し方（さくら町）
 月・木：もえる ゴミ
 火：プラスチック
 水：びん・かん
 金：古い 紙
 ※朝 8時までに 出して ください。
+━━━━━━━━━━━━━━━━━━
 (1) びんは 何曜日に 出しますか。</t>
         </is>
       </c>
@@ -2607,12 +2625,14 @@
       <c r="B47" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 ゴミの 出し方（さくら町）
 月・木：もえる ゴミ
 火：プラスチック
 水：びん・かん
 金：古い 紙
 ※朝 8時までに 出して ください。
+━━━━━━━━━━━━━━━━━━
 (2) ゴミは 何時までに 出しますか。</t>
         </is>
       </c>
@@ -2655,11 +2675,13 @@
       <c r="B48" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 さくら市 体育館
 開館時間：9:00～21:00
 休館日：毎週 月曜日
 りよう料金：大人 300円　子ども 100円
 ※中では 運動ぐつを はいて ください。
+━━━━━━━━━━━━━━━━━━
 (1) 体育館が 休みの 日は 何曜日ですか。</t>
         </is>
       </c>
@@ -2702,11 +2724,13 @@
       <c r="B49" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
+━━━━━━ BÀI ĐỌC ━━━━━━
 さくら市 体育館
 開館時間：9:00～21:00
 休館日：毎週 月曜日
 りよう料金：大人 300円　子ども 100円
 ※中では 運動ぐつを はいて ください。
+━━━━━━━━━━━━━━━━━━
 (2) 大人 2人と 子ども 1人で いくらですか。</t>
         </is>
       </c>

</xml_diff>

<commit_message>
DF-01: điền Image Url 16 tranh từ Drive
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011epdNWjc77FA9dxPqBsa8Z
</commit_message>
<xml_diff>
--- a/exports/DF-01_LMS_import.xlsx
+++ b/exports/DF-01_LMS_import.xlsx
@@ -478,7 +478,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Nhìn hình và chọn một từ phù hợp nhất.
@@ -495,7 +494,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JQ-0025.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=14iuyB1ioqdq_M4rhK_ZOYOAD8oL6UKEy</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -513,7 +512,6 @@
           <t>かさ</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
         <v>1</v>
       </c>
@@ -524,7 +522,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Nhìn hình và chọn một từ phù hợp nhất.
@@ -541,7 +538,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>JQ-0026.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1bhzjZ3nxbchCx3FxKDOk09t7VB5fEvrI</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -559,7 +556,6 @@
           <t>タクシー</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
         <v>2</v>
       </c>
@@ -570,7 +566,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>Nhìn hình và chọn một từ phù hợp nhất.
@@ -587,7 +582,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>JQ-0027.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=138pbQ0rVJ0xc5lPDp1qR6MibMuM8eYpX</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -605,7 +600,6 @@
           <t>せんたく</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
         <v>3</v>
       </c>
@@ -616,7 +610,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Nhìn hình và chọn một từ phù hợp nhất.
@@ -633,7 +626,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>JQ-0028.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1hmru7MU5s78d6MTBpDjGdeyhNkt3FUSV</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -651,7 +644,6 @@
           <t>とけい</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
         <v>4</v>
       </c>
@@ -662,7 +654,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Đọc câu và chọn từ phù hợp nhất để điền vào chỗ trống.
@@ -678,7 +669,6 @@
           <t>Trời mưa nên mang ô → かさ.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>めがね</t>
@@ -694,7 +684,6 @@
           <t>さいふ</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
         <v>5</v>
       </c>
@@ -705,7 +694,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Đọc câu và chọn từ phù hợp nhất để điền vào chỗ trống.
@@ -721,7 +709,6 @@
           <t>Phòng tối nên "bật" đèn → つけて. けして: tắt; しめて: đóng.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>つけて</t>
@@ -737,7 +724,6 @@
           <t>しめて</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
         <v>6</v>
       </c>
@@ -748,7 +734,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Đọc câu và chọn từ phù hợp nhất để điền vào chỗ trống.
@@ -764,7 +749,6 @@
           <t>Bị sốt nên "nghỉ" làm → やすみます.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>はたらきます</t>
@@ -780,7 +764,6 @@
           <t>やすみます</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
         <v>7</v>
       </c>
@@ -791,7 +774,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Chọn cách đọc bằng hiragana đúng của từ trong 【　】.
@@ -807,7 +789,6 @@
           <t>毎日 đọc là まいにち (mỗi ngày).</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>まいにち</t>
@@ -823,7 +804,6 @@
           <t>まいじつ</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
         <v>8</v>
       </c>
@@ -834,7 +814,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>Chọn cách đọc bằng hiragana đúng của từ trong 【　】.
@@ -850,7 +829,6 @@
           <t>前 đứng một mình (phía trước) đọc là まえ; ぜん là âm On dùng trong từ ghép.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>ぜん</t>
@@ -866,7 +844,6 @@
           <t>まい</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
         <v>9</v>
       </c>
@@ -877,7 +854,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>Chọn cách đọc bằng hiragana đúng của từ trong 【　】.
@@ -893,7 +869,6 @@
           <t>休み đọc là やすみ (ngày nghỉ).</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>よすみ</t>
@@ -909,7 +884,6 @@
           <t>やすみ</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
         <v>10</v>
       </c>
@@ -920,7 +894,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>Đọc câu và chọn từ viết bằng chữ Hán phù hợp nhất để điền vào chỗ trống.
@@ -936,7 +909,6 @@
           <t>Cà phê thì "uống" → 飲みます.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>食べます</t>
@@ -952,7 +924,6 @@
           <t>書きます</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="n">
         <v>11</v>
       </c>
@@ -963,7 +934,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>Đọc câu và chọn từ viết bằng chữ Hán phù hợp nhất để điền vào chỗ trống.
@@ -979,7 +949,6 @@
           <t>Mẹ "làm việc" ở bệnh viện → 働いています. 住んでいます đi với に.</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>働いて います</t>
@@ -995,7 +964,6 @@
           <t>住んで います</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="n">
         <v>12</v>
       </c>
@@ -1006,7 +974,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn phương án phù hợp nhất để điền vào chỗ trống.
@@ -1023,7 +990,6 @@
           <t>Nối hai hành động theo thứ tự: V-て、V2. 〜たり phải đi thành cặp 〜たり〜たりしました.</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>たり</t>
@@ -1054,7 +1020,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn phương án phù hợp nhất để điền vào chỗ trống.
@@ -1071,7 +1036,6 @@
           <t>まだ + phủ định hiện tại: "vẫn chưa đọc được" → 読めません.</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>ました</t>
@@ -1102,7 +1066,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn phương án phù hợp nhất để điền vào chỗ trống.
@@ -1119,7 +1082,6 @@
           <t>Khuyên: V-たほうがいい.</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>ほう</t>
@@ -1150,7 +1112,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn phương án phù hợp nhất để điền vào chỗ trống.
@@ -1167,7 +1128,6 @@
           <t>Người/động vật tồn tại dùng います.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>あります</t>
@@ -1198,7 +1158,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn phương án phù hợp nhất để điền vào chỗ trống.
@@ -1215,7 +1174,6 @@
           <t>Điều kiện "nếu mưa thì…" → 〜たら.</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>ながら</t>
@@ -1246,7 +1204,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn phương án phù hợp nhất để điền vào chỗ trống.
@@ -1263,7 +1220,6 @@
           <t>Người khác làm cho mình → V-てくれました.</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>くれました</t>
@@ -1294,7 +1250,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn lời nói hoặc lời đáp phù hợp nhất để điền vào chỗ trống.
@@ -1312,7 +1267,6 @@
           <t>Đến muộn → xin lỗi. おつかれさまでした dùng khi chia tay sau giờ làm; いってきます khi rời nhà.</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>おそく なって、すみません。</t>
@@ -1328,7 +1282,6 @@
           <t>いってきます。</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="n">
         <v>19</v>
       </c>
@@ -1339,7 +1292,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn lời nói hoặc lời đáp phù hợp nhất để điền vào chỗ trống.
@@ -1356,7 +1308,6 @@
           <t>Gọi món với nhân viên: N を おねがいします.</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>カレーは どうですか。</t>
@@ -1372,7 +1323,6 @@
           <t>カレーを おねがいします。</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="n">
         <v>20</v>
       </c>
@@ -1383,7 +1333,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn lời nói hoặc lời đáp phù hợp nhất để điền vào chỗ trống.
@@ -1400,7 +1349,6 @@
           <t>Đáp lời đồng nghiệp về trước: おつかれさまでした.</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>いってらっしゃい。</t>
@@ -1416,7 +1364,6 @@
           <t>おかえりなさい。</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="n">
         <v>21</v>
       </c>
@@ -1427,7 +1374,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn lời nói hoặc lời đáp phù hợp nhất để điền vào chỗ trống.
@@ -1444,7 +1390,6 @@
           <t>Nhận lời mời: いいですね。〜ましょう.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>いいですね。行きましょう。</t>
@@ -1460,7 +1405,6 @@
           <t>はい、見に 行きました。</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="n">
         <v>22</v>
       </c>
@@ -1471,7 +1415,6 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn lời nói hoặc lời đáp phù hợp nhất để điền vào chỗ trống.
@@ -1488,7 +1431,6 @@
           <t>Chưa nghe rõ → nhờ nói lại: もう一度おねがいします.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>どういたしまして。</t>
@@ -1504,7 +1446,6 @@
           <t>すみません、もう 一度 おねがいします。</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
         <v>23</v>
       </c>
@@ -1515,7 +1456,6 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
           <t>Đọc hội thoại và chọn lời nói hoặc lời đáp phù hợp nhất để điền vào chỗ trống.
@@ -1532,7 +1472,6 @@
           <t>Hỏi thăm khi người khác không khoẻ.</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>よかったですね。</t>
@@ -1548,7 +1487,6 @@
           <t>おめでとうございます。</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="n">
         <v>24</v>
       </c>
@@ -1581,7 +1519,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>JQ-0049.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1bSX2wAZ0Yd-AdeODq89fNM-PYCysG7ug</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1599,7 +1537,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="n">
         <v>25</v>
       </c>
@@ -1632,7 +1569,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>JQ-0050.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1CdZlHgqgUBowat4ypMjU8PSsvndW1IxU</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1650,7 +1587,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="n">
         <v>26</v>
       </c>
@@ -1683,7 +1619,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>JQ-0051.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1vn_KHkMtbxL48QN1MI4_4v6ckq27DE0L</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1701,7 +1637,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="n">
         <v>27</v>
       </c>
@@ -1734,7 +1669,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>JQ-0052.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1b_w2mG1bQg2Zd9-xv1XyttZvVvfE5cJf</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1752,7 +1687,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="n">
         <v>28</v>
       </c>
@@ -1785,7 +1719,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>JQ-0053.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1--cEZGFB3liGvYUGTVlDP8ABO2KQAGIt</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1803,7 +1737,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="n">
         <v>29</v>
       </c>
@@ -1836,7 +1769,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>JQ-0054.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1gjzhCQbaM3TDx3Ua7YcAlc71nSX1xweJ</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1854,7 +1787,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="n">
         <v>30</v>
       </c>
@@ -1887,7 +1819,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>JQ-0055.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1myUWSBGK-7DrM1C-ISd-_uE9q_90jGVO</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1905,7 +1837,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" t="n">
         <v>31</v>
       </c>
@@ -1938,7 +1869,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>JQ-0056.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1KC0s65nI7YSTzf7eDrf8hIElQFrgjyWQ</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1956,7 +1887,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="n">
         <v>32</v>
       </c>
@@ -1991,7 +1921,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>JQ-0057.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1GdsmG-oth7cMBUeXpSfSzgFeGQ0M7neF</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2009,7 +1939,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="n">
         <v>33</v>
       </c>
@@ -2044,7 +1973,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>JQ-0058.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1J9WHgJbSiCXBiN4a2vUmwHw174i1_wHw</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2062,7 +1991,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="n">
         <v>34</v>
       </c>
@@ -2097,7 +2025,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>JQ-0059.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1Qvg1awZeEbQ_ZoCEiQs9DG14lReqcX-k</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2115,7 +2043,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="n">
         <v>35</v>
       </c>
@@ -2150,7 +2077,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>JQ-0060.png</t>
+          <t>https://drive.google.com/uc?export=view&amp;id=1rhcts7JhYF2q64cqTDNZJFya-Kdjo7Uu</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2168,7 +2095,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" t="n">
         <v>36</v>
       </c>
@@ -2179,7 +2105,6 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
@@ -2200,7 +2125,6 @@
           <t>"ねつが あって、きょうは 会社を 休みたいです".</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>いそがしいから</t>
@@ -2216,7 +2140,6 @@
           <t>たなかさんが 休むから</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="n">
         <v>37</v>
       </c>
@@ -2227,7 +2150,6 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
@@ -2248,7 +2170,6 @@
           <t>"あしたは 来られると 思います".</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>きのう</t>
@@ -2264,7 +2185,6 @@
           <t>あした</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" t="n">
         <v>38</v>
       </c>
@@ -2275,7 +2195,6 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
@@ -2296,7 +2215,6 @@
           <t>"家族と すいぞくかんに 行きました".</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>家族</t>
@@ -2312,7 +2230,6 @@
           <t>会社の 人</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="n">
         <v>39</v>
       </c>
@@ -2323,7 +2240,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
@@ -2344,7 +2260,6 @@
           <t>"むすこは ペンギンが いちばん 好きだと".</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>イルカ</t>
@@ -2360,7 +2275,6 @@
           <t>ショー</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="n">
         <v>40</v>
       </c>
@@ -2371,7 +2285,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
@@ -2393,7 +2306,6 @@
           <t>Trước 10 giờ mang hộp lên kho, "そのあと" mới xếp ghế.</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>会議に 出る</t>
@@ -2409,7 +2321,6 @@
           <t>はこを 運ぶ</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
       <c r="J42" t="n">
         <v>41</v>
       </c>
@@ -2420,7 +2331,6 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
           <t>Đọc bài và trả lời câu hỏi (1) và (2).
@@ -2442,7 +2352,6 @@
           <t>"11時から 会議が あります".</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>10時</t>
@@ -2458,7 +2367,6 @@
           <t>2時</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="n">
         <v>42</v>
       </c>
@@ -2469,7 +2377,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
@@ -2493,7 +2400,6 @@
           <t>Chỉ ぎゅうどん 550円 ≤ 600円.</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>カレー</t>
@@ -2509,7 +2415,6 @@
           <t>ぎゅうどん</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
       <c r="J44" t="n">
         <v>43</v>
       </c>
@@ -2520,7 +2425,6 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
@@ -2544,7 +2448,6 @@
           <t>"ランチは 11:00～14:00" → đến 14 giờ.</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>14時</t>
@@ -2560,7 +2463,6 @@
           <t>16時</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
       <c r="J45" t="n">
         <v>44</v>
       </c>
@@ -2571,7 +2473,6 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
@@ -2594,7 +2495,6 @@
           <t>"水：びん・かん" → thứ Tư.</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>月曜日</t>
@@ -2610,7 +2510,6 @@
           <t>金曜日</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
       <c r="J46" t="n">
         <v>45</v>
       </c>
@@ -2621,7 +2520,6 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
@@ -2644,7 +2542,6 @@
           <t>"朝 8時までに".</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>7時</t>
@@ -2660,7 +2557,6 @@
           <t>8時</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
       <c r="J47" t="n">
         <v>46</v>
       </c>
@@ -2671,7 +2567,6 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
@@ -2693,7 +2588,6 @@
           <t>"休館日：毎週 月曜日".</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>月曜日</t>
@@ -2709,7 +2603,6 @@
           <t>日曜日</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
       <c r="J48" t="n">
         <v>47</v>
       </c>
@@ -2720,7 +2613,6 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
           <t>Đọc thông tin và trả lời câu hỏi (1) và (2).
@@ -2742,7 +2634,6 @@
           <t>300×2 + 100 = 700円.</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>400円</t>
@@ -2758,7 +2649,6 @@
           <t>700円</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
       <c r="J49" t="n">
         <v>48</v>
       </c>

</xml_diff>

<commit_message>
DF-01: điền Audio Url (S3) cho 12 câu nghe
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FV5t8ch9TrTXwKKVmMzCy5
</commit_message>
<xml_diff>
--- a/exports/DF-01_LMS_import.xlsx
+++ b/exports/DF-01_LMS_import.xlsx
@@ -1499,7 +1499,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AUDIO_JQ-0049.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920089-audio_jq-0049wav</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1549,7 +1549,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AUDIO_JQ-0050.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_jq-0050wav</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1599,7 +1599,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AUDIO_JQ-0051.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_jq-0051wav</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1649,7 +1649,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AUDIO_JQ-0052.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_jq-0052wav</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1699,7 +1699,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AUDIO_JQ-0053.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_jq-0053wav</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1749,7 +1749,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AUDIO_JQ-0054.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_jq-0054wav</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1799,7 +1799,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AUDIO_JQ-0055.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_jq-0055wav</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1849,7 +1849,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AUDIO_JQ-0056.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_jq-0056wav</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1899,7 +1899,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AUDIO_G-0005.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_g-0005wav</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1951,7 +1951,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AUDIO_G-0005.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_g-0005wav</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2003,7 +2003,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AUDIO_G-0006.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_g-0006wav</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2055,7 +2055,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AUDIO_G-0006.wav</t>
+          <t>https://rikkeiedu-storage.s3.ap-southeast-2.amazonaws.com/uploads/1791570920088-audio_g-0006wav</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">

</xml_diff>